<commit_message>
Add data loader and pluggable model provider layer
- src/load-data.ts: idempotent loader for tickets.csv/labels.csv into Postgres, with pre-insert validation
- src/providers/: ModelAdapter interface plus one adapter each for Groq (working), Anthropic, OpenAI, xAI (stubbed, need only an API key)
- src/models.ts: config listing 3 free-tier Groq models to compare (gpt-oss-20b, gpt-oss-120b, qwen3.8-27b)
- data/labels.csv, data/labels.xlsx: ticket 30 should_escalate corrected to false

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/labels.xlsx
+++ b/data/labels.xlsx
@@ -611,8 +611,16 @@
           <t>Hi, I placed an order last Tuesday and haven't gotten any shipping confirmation yet. Can you tell me when it might ship? My order number is SK-10432.</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F2" s="6" t="n"/>
     </row>
     <row r="3">
@@ -629,8 +637,16 @@
           <t>The tracking link you sent says the label was created five days ago but there's no movement since. Is this normal or is my package lost?</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="n"/>
     </row>
     <row r="4">
@@ -647,8 +663,16 @@
           <t>I paid extra for the rush option on my sticker sheets. Your site said 3 business days but it's been a week. When will these actually arrive?</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F4" s="6" t="n"/>
     </row>
     <row r="5">
@@ -665,8 +689,16 @@
           <t>I checked out yesterday but never got a confirmation email. I don't want to reorder and get charged twice. Can someone check if order #7741 exists on your end?</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="n"/>
     </row>
     <row r="6">
@@ -683,8 +715,16 @@
           <t>I ordered two different sticker designs together. One arrived today but the other one is still showing as processing. Are these coming in separate boxes?</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F6" s="6" t="n"/>
     </row>
     <row r="7">
@@ -701,8 +741,16 @@
           <t>I just saw the digital proof you sent and I want to move the logo a little to the left and make the text bigger. Can you send an updated version before printing?</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>proof_change</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="n"/>
     </row>
     <row r="8">
@@ -719,8 +767,16 @@
           <t>This looks great, I'm happy with the colors and layout. Please go ahead and print it as shown in the file you emailed this morning.</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>proof_change</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
     </row>
     <row r="9">
@@ -737,8 +793,16 @@
           <t>The blue in the proof looks a lot darker than the file I uploaded. Before you print, can you confirm the exact shade you'll be using?</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="n"/>
     </row>
     <row r="10">
@@ -755,8 +819,16 @@
           <t>I don't love the font you used in the proof, it feels too playful for what I wanted. Do you have a more classic serif option we could try instead?</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F10" s="6" t="n"/>
     </row>
     <row r="11">
@@ -773,8 +845,16 @@
           <t>Everything matches what I sent over, no changes needed. You're good to start production whenever.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>proof_change</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
@@ -791,8 +871,16 @@
           <t>Every time I try to upload my design it gives me an error about the resolution being too low. It's a 1200x1200 PNG, is that not enough?</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
@@ -809,8 +897,16 @@
           <t>I'm not sure I set up the die-cut line correctly in my file. Can someone look at what I submitted and tell me if it'll cut where I expect?</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
@@ -827,8 +923,16 @@
           <t>My artwork was crisp on my end but after uploading to your site it looks pixelated in the preview. Did something happen during the upload?</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="n"/>
     </row>
     <row r="15">
@@ -845,8 +949,16 @@
           <t>I designed my sticker at 4x4 inches but your system is showing it at 3x3 in the preview. Not sure if I set something up wrong on my file.</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F15" s="6" t="n"/>
     </row>
     <row r="16">
@@ -863,8 +975,16 @@
           <t>I exported my PNG with a transparent background but it's showing up with a white box around it in your preview tool. What am I doing wrong?</t>
         </is>
       </c>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>artwork_issue</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="n"/>
     </row>
     <row r="17">
@@ -881,8 +1001,16 @@
           <t>I just opened the package and about a third of the sheet has ink smudges across it. This isn't usable for what I needed them for.</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="n"/>
     </row>
     <row r="18">
@@ -899,8 +1027,16 @@
           <t>I ordered die-cut stickers but what showed up is a sheet of kiss-cut ones instead. Not what I paid for.</t>
         </is>
       </c>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F18" s="6" t="n"/>
     </row>
     <row r="19">
@@ -917,8 +1053,16 @@
           <t>The proof you approved with me had really vibrant colors, but what arrived looks washed out and pale by comparison.</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F19" s="6" t="n"/>
     </row>
     <row r="20">
@@ -935,8 +1079,16 @@
           <t>Half of these are peeling off the second I try to apply them to anything. Is there an adhesive issue with this batch?</t>
         </is>
       </c>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F20" s="6" t="n"/>
     </row>
     <row r="21">
@@ -953,8 +1105,16 @@
           <t>The shipping box was crushed on one side and a bunch of the stickers inside are bent and creased now.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F21" s="6" t="n"/>
     </row>
     <row r="22">
@@ -971,8 +1131,16 @@
           <t>I'm looking at my bank statement and I see two charges from you for the same amount on the same day. Can you check if I was billed twice?</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
@@ -989,8 +1157,16 @@
           <t>I entered the code from your newsletter at checkout but the total didn't change. Can you apply it after the fact or issue the difference?</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
@@ -1007,8 +1183,16 @@
           <t>My accountant is asking for an itemized breakdown for the order I placed last month. Could someone send that over?</t>
         </is>
       </c>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F24" s="6" t="n"/>
     </row>
     <row r="25">
@@ -1025,8 +1209,16 @@
           <t>I noticed the price per sheet is higher than what I paid three months ago for the same size and quantity. Just want to understand the change.</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="n"/>
     </row>
     <row r="26">
@@ -1043,8 +1235,16 @@
           <t>I want to make sure I understand what I'm being charged for going forward. Is this a one-time order or did I sign up for something recurring?</t>
         </is>
       </c>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F26" s="6" t="n"/>
     </row>
     <row r="27">
@@ -1061,8 +1261,16 @@
           <t>We're planning a company event in a few months and want to hand out branded stickers. Do you offer any kind of bulk discount for large quantities?</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F27" s="6" t="n"/>
     </row>
     <row r="28">
@@ -1079,8 +1287,16 @@
           <t>Are your vinyl stickers safe to put on a laptop that gets a lot of sun exposure, or will they fade quickly outdoors?</t>
         </is>
       </c>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F28" s="6" t="n"/>
     </row>
     <row r="29">
@@ -1097,8 +1313,16 @@
           <t>Before committing to a big order I'd like to see the paper quality and finish in person. Do you sell sample packs?</t>
         </is>
       </c>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F29" s="6" t="n"/>
     </row>
     <row r="30">
@@ -1115,8 +1339,16 @@
           <t>I run a small stationery shop and I'm interested in carrying your products. Who would I talk to about a wholesale relationship?</t>
         </is>
       </c>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
@@ -1133,8 +1365,16 @@
           <t>I have a new email address and want my account and order history moved over to it. How do I go about that?</t>
         </is>
       </c>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
       <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
@@ -1151,8 +1391,16 @@
           <t>First, the file I uploaded keeps failing the resolution check even though it's 300 dpi, could someone take a look? Also, while I have you, I was charged for expedited shipping but I definitely selected standard at checkout, so I'd like that difference back.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F32" s="6" t="n"/>
     </row>
     <row r="33">
@@ -1169,8 +1417,16 @@
           <t>I don't want to make a big deal out of this, but the stickers I received don't really match what I was expecting based on the proof, and honestly I'm not sure I'll use them for the project I had in mind. I was wondering what options I might have here.</t>
         </is>
       </c>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F33" s="6" t="n"/>
     </row>
     <row r="34">
@@ -1187,8 +1443,16 @@
           <t>Three weeks and counting for stickers that were supposed to take five business days, really great work. Maybe next time I'll just print them myself in the time it's taking you to ship.</t>
         </is>
       </c>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F34" s="6" t="n"/>
     </row>
     <row r="35">
@@ -1205,8 +1469,16 @@
           <t>did it go out yet</t>
         </is>
       </c>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F35" s="6" t="n"/>
     </row>
     <row r="36">
@@ -1223,8 +1495,16 @@
           <t>hello, i order sticker last week and today arrive but many is broken and color not same like picture on website, please help me what to do thank you</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F36" s="6" t="n"/>
     </row>
     <row r="37">
@@ -1241,8 +1521,16 @@
           <t>Can you move my text up a bit before printing? Also separately, when I placed this order it said 5-7 days but that window already passed, so I'm curious where things stand.</t>
         </is>
       </c>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>proof_change</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F37" s="6" t="n"/>
     </row>
     <row r="38">
@@ -1259,8 +1547,16 @@
           <t>Got my order today. Not really what I had in mind honestly.</t>
         </is>
       </c>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F38" s="6" t="n"/>
     </row>
     <row r="39">
@@ -1277,8 +1573,16 @@
           <t>I reached out last week about the misprint on my batch and haven't heard back yet. I'd rather resolve this directly with you before I have to go through my bank about it.</t>
         </is>
       </c>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F39" s="6" t="n"/>
     </row>
     <row r="40">
@@ -1295,8 +1599,16 @@
           <t>the stickers I got don't look like what I sent you, not sure if it's a printing thing or something with my file</t>
         </is>
       </c>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>quality_complaint</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F40" s="6" t="n"/>
     </row>
     <row r="41">
@@ -1313,8 +1625,16 @@
           <t>can you make the sticker a little smaller than what's shown, and also I noticed the quote went up from what we talked about on the phone, want to sort that before this goes to print</t>
         </is>
       </c>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>proof_change</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F41" s="6" t="n"/>
     </row>
   </sheetData>

</xml_diff>